<commit_message>
Add 詳細 column to フェーズ管理 Tier feature list
Each of the 23 features (F-01 to F-23) now has a detailed description
explaining exactly what the feature does, how it works, and what data
it interacts with. Row height set to 60px for readability.

Examples:
- F-07: "工務店一覧で最大3社にチェック→1回のフォーム送信で3社同時に資料請求..."
- F-08: "eventsにcapacity/reserved_countを追加。残り○組バッジ表示..."
- F-12: "リード発生後9通の自動配信。3ヶ月後のアンケートで成約把握率50%→85%..."

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/05_プロジェクト管理/PFプロジェクト管理表.xlsx
+++ b/docs/05_プロジェクト管理/PFプロジェクト管理表.xlsx
@@ -198,7 +198,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -322,11 +322,12 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -464,6 +465,8 @@
     <xf numFmtId="0" fontId="13" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1517,18 +1520,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -1538,6 +1541,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="26" t="inlineStr">
         <is>
@@ -1755,6 +1759,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
         <is>
@@ -2279,6 +2284,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
         <is>
@@ -2803,6 +2809,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
         <is>
@@ -3186,6 +3193,8 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="26" t="inlineStr">
         <is>
@@ -3517,12 +3526,27 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="51" t="inlineStr">
+      <c r="A62" s="57" t="inlineStr">
         <is>
           <t>【収益ドリブン機能とフェーズの紐付け】</t>
         </is>
       </c>
+      <c r="B62" s="58" t="n"/>
+      <c r="C62" s="58" t="n"/>
+      <c r="D62" s="58" t="n"/>
+      <c r="E62" s="58" t="n"/>
+      <c r="F62" s="58" t="n"/>
+      <c r="G62" s="58" t="n"/>
+      <c r="H62" s="58" t="n"/>
+      <c r="I62" s="58" t="n"/>
+      <c r="J62" s="58" t="n"/>
+      <c r="K62" s="58" t="n"/>
+      <c r="L62" s="58" t="n"/>
+      <c r="M62" s="58" t="n"/>
+      <c r="N62" s="58" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
@@ -3552,21 +3576,31 @@
       </c>
       <c r="F63" s="27" t="inlineStr">
         <is>
+          <t>詳細</t>
+        </is>
+      </c>
+      <c r="G63" s="27" t="inlineStr">
+        <is>
           <t>売上インパクト</t>
         </is>
       </c>
-      <c r="G63" s="27" t="inlineStr">
+      <c r="H63" s="27" t="inlineStr">
         <is>
           <t>開発工数</t>
         </is>
       </c>
-      <c r="H63" s="27" t="inlineStr">
+      <c r="I63" s="27" t="inlineStr">
         <is>
           <t>ステータス</t>
         </is>
       </c>
-    </row>
-    <row r="64">
+      <c r="J63" s="58" t="n"/>
+      <c r="K63" s="58" t="n"/>
+      <c r="L63" s="58" t="n"/>
+      <c r="M63" s="58" t="n"/>
+      <c r="N63" s="58" t="n"/>
+    </row>
+    <row r="64" ht="60" customHeight="1">
       <c r="A64" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3579,7 +3613,7 @@
       </c>
       <c r="C64" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D64" s="53" t="inlineStr">
@@ -3592,23 +3626,33 @@
           <t>資料請求フォーム本番稼働</t>
         </is>
       </c>
-      <c r="F64" s="53" t="inlineStr">
+      <c r="F64" s="28" t="inlineStr">
+        <is>
+          <t>消費者が工務店を選んで資料請求→工務店にメール通知→Supabaseにリード保存。本番環境での送信テスト・通知到達確認が必須</t>
+        </is>
+      </c>
+      <c r="G64" s="53" t="inlineStr">
         <is>
           <t>年間1,440万円の基盤</t>
         </is>
       </c>
-      <c r="G64" s="53" t="inlineStr">
+      <c r="H64" s="53" t="inlineStr">
         <is>
           <t>済</t>
         </is>
       </c>
-      <c r="H64" s="53" t="inlineStr">
+      <c r="I64" s="53" t="inlineStr">
         <is>
           <t>✅ 実装済</t>
         </is>
       </c>
-    </row>
-    <row r="65">
+      <c r="J64" s="58" t="n"/>
+      <c r="K64" s="58" t="n"/>
+      <c r="L64" s="58" t="n"/>
+      <c r="M64" s="58" t="n"/>
+      <c r="N64" s="58" t="n"/>
+    </row>
+    <row r="65" ht="60" customHeight="1">
       <c r="A65" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3621,7 +3665,7 @@
       </c>
       <c r="C65" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D65" s="53" t="inlineStr">
@@ -3634,23 +3678,33 @@
           <t>見学会予約フォーム本番稼働</t>
         </is>
       </c>
-      <c r="F65" s="53" t="inlineStr">
+      <c r="F65" s="28" t="inlineStr">
+        <is>
+          <t>消費者が見学会を選んで予約→工務店にメール通知→予約数カウント更新。最大の収益源（1件8万円）のため確実な動作が最重要</t>
+        </is>
+      </c>
+      <c r="G65" s="53" t="inlineStr">
         <is>
           <t>年間6,720万円の基盤</t>
         </is>
       </c>
-      <c r="G65" s="53" t="inlineStr">
+      <c r="H65" s="53" t="inlineStr">
         <is>
           <t>済</t>
         </is>
       </c>
-      <c r="H65" s="53" t="inlineStr">
+      <c r="I65" s="53" t="inlineStr">
         <is>
           <t>✅ 実装済</t>
         </is>
       </c>
-    </row>
-    <row r="66">
+      <c r="J65" s="58" t="n"/>
+      <c r="K65" s="58" t="n"/>
+      <c r="L65" s="58" t="n"/>
+      <c r="M65" s="58" t="n"/>
+      <c r="N65" s="58" t="n"/>
+    </row>
+    <row r="66" ht="60" customHeight="1">
       <c r="A66" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3663,7 +3717,7 @@
       </c>
       <c r="C66" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D66" s="53" t="inlineStr">
@@ -3676,23 +3730,33 @@
           <t>無料相談フォーム本番稼働</t>
         </is>
       </c>
-      <c r="F66" s="53" t="inlineStr">
+      <c r="F66" s="28" t="inlineStr">
+        <is>
+          <t>氏名・電話・メール・相談内容を入力して送信。相談リードは将来の見学会参加・成約につながる入口</t>
+        </is>
+      </c>
+      <c r="G66" s="53" t="inlineStr">
         <is>
           <t>リード獲得の入口</t>
         </is>
       </c>
-      <c r="G66" s="53" t="inlineStr">
+      <c r="H66" s="53" t="inlineStr">
         <is>
           <t>済</t>
         </is>
       </c>
-      <c r="H66" s="53" t="inlineStr">
+      <c r="I66" s="53" t="inlineStr">
         <is>
           <t>✅ 実装済</t>
         </is>
       </c>
-    </row>
-    <row r="67">
+      <c r="J66" s="58" t="n"/>
+      <c r="K66" s="58" t="n"/>
+      <c r="L66" s="58" t="n"/>
+      <c r="M66" s="58" t="n"/>
+      <c r="N66" s="58" t="n"/>
+    </row>
+    <row r="67" ht="60" customHeight="1">
       <c r="A67" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3705,7 +3769,7 @@
       </c>
       <c r="C67" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D67" s="53" t="inlineStr">
@@ -3718,23 +3782,33 @@
           <t>50社分の実データ投入</t>
         </is>
       </c>
-      <c r="F67" s="53" t="inlineStr">
+      <c r="F67" s="28" t="inlineStr">
+        <is>
+          <t>50社の企業情報・施工事例写真3〜5枚・坪単価・対応エリア・平屋実績・デザインテイスト・強みをCMS管理画面から入力。掲載基準ガイドに基づく品質統一</t>
+        </is>
+      </c>
+      <c r="G67" s="53" t="inlineStr">
         <is>
           <t>全収益の前提</t>
         </is>
       </c>
-      <c r="G67" s="53" t="inlineStr">
+      <c r="H67" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H67" s="53" t="inlineStr">
+      <c r="I67" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="68">
+      <c r="J67" s="58" t="n"/>
+      <c r="K67" s="58" t="n"/>
+      <c r="L67" s="58" t="n"/>
+      <c r="M67" s="58" t="n"/>
+      <c r="N67" s="58" t="n"/>
+    </row>
+    <row r="68" ht="60" customHeight="1">
       <c r="A68" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3747,7 +3821,7 @@
       </c>
       <c r="C68" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D68" s="53" t="inlineStr">
@@ -3760,23 +3834,33 @@
           <t>リード通知メール本番稼働</t>
         </is>
       </c>
-      <c r="F68" s="53" t="inlineStr">
+      <c r="F68" s="28" t="inlineStr">
+        <is>
+          <t>Resend APIで工務店担当者に即時通知。件名・本文にリード情報（氏名・連絡先・問い合わせ内容・閲覧履歴）を含める</t>
+        </is>
+      </c>
+      <c r="G68" s="53" t="inlineStr">
         <is>
           <t>工務店信頼に直結</t>
         </is>
       </c>
-      <c r="G68" s="53" t="inlineStr">
+      <c r="H68" s="53" t="inlineStr">
         <is>
           <t>3日</t>
         </is>
       </c>
-      <c r="H68" s="53" t="inlineStr">
+      <c r="I68" s="53" t="inlineStr">
         <is>
           <t>✅ 実装済</t>
         </is>
       </c>
-    </row>
-    <row r="69">
+      <c r="J68" s="58" t="n"/>
+      <c r="K68" s="58" t="n"/>
+      <c r="L68" s="58" t="n"/>
+      <c r="M68" s="58" t="n"/>
+      <c r="N68" s="58" t="n"/>
+    </row>
+    <row r="69" ht="60" customHeight="1">
       <c r="A69" s="52" t="inlineStr">
         <is>
           <t>Tier 1</t>
@@ -3789,7 +3873,7 @@
       </c>
       <c r="C69" s="53" t="inlineStr">
         <is>
-          <t>5月リリース前</t>
+          <t>5月前</t>
         </is>
       </c>
       <c r="D69" s="53" t="inlineStr">
@@ -3802,23 +3886,33 @@
           <t>AIチャット本番稼働</t>
         </is>
       </c>
-      <c r="F69" s="53" t="inlineStr">
+      <c r="F69" s="28" t="inlineStr">
+        <is>
+          <t>GPT-4oのプロンプトに50社の工務店情報を反映。FAQ回答精度の検証。月間APIコスト上限$100の設定確認</t>
+        </is>
+      </c>
+      <c r="G69" s="53" t="inlineStr">
         <is>
           <t>相談→リード化</t>
         </is>
       </c>
-      <c r="G69" s="53" t="inlineStr">
+      <c r="H69" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H69" s="53" t="inlineStr">
+      <c r="I69" s="53" t="inlineStr">
         <is>
           <t>✅ 実装済</t>
         </is>
       </c>
-    </row>
-    <row r="70">
+      <c r="J69" s="58" t="n"/>
+      <c r="K69" s="58" t="n"/>
+      <c r="L69" s="58" t="n"/>
+      <c r="M69" s="58" t="n"/>
+      <c r="N69" s="58" t="n"/>
+    </row>
+    <row r="70" ht="60" customHeight="1">
       <c r="A70" s="54" t="inlineStr">
         <is>
           <t>Tier 2</t>
@@ -3844,23 +3938,33 @@
           <t>まとめて資料請求（3社一括）</t>
         </is>
       </c>
-      <c r="F70" s="53" t="inlineStr">
+      <c r="F70" s="28" t="inlineStr">
+        <is>
+          <t>工務店一覧で最大3社にチェック→1回のフォーム送信で3社同時に資料請求。各社にリード通知メールを個別送信。leadsテーブルに1社1レコード作成。資料請求件数が3倍になる最高ROI機能</t>
+        </is>
+      </c>
+      <c r="G70" s="53" t="inlineStr">
         <is>
           <t>年間+960万円</t>
         </is>
       </c>
-      <c r="G70" s="53" t="inlineStr">
+      <c r="H70" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H70" s="53" t="inlineStr">
+      <c r="I70" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="71">
+      <c r="J70" s="58" t="n"/>
+      <c r="K70" s="58" t="n"/>
+      <c r="L70" s="58" t="n"/>
+      <c r="M70" s="58" t="n"/>
+      <c r="N70" s="58" t="n"/>
+    </row>
+    <row r="71" ht="60" customHeight="1">
       <c r="A71" s="54" t="inlineStr">
         <is>
           <t>Tier 2</t>
@@ -3886,23 +3990,33 @@
           <t>見学会残席表示＋今週末特集</t>
         </is>
       </c>
-      <c r="F71" s="53" t="inlineStr">
+      <c r="F71" s="28" t="inlineStr">
+        <is>
+          <t>eventsにcapacity/reserved_countを追加。「残り○組」バッジ表示。残席3以下で「残りわずか」、0で「満席」。TOPに「今週末の見学会」セクション自動表示</t>
+        </is>
+      </c>
+      <c r="G71" s="53" t="inlineStr">
         <is>
           <t>年間+1,920万円</t>
         </is>
       </c>
-      <c r="G71" s="53" t="inlineStr">
+      <c r="H71" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H71" s="53" t="inlineStr">
+      <c r="I71" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="72">
+      <c r="J71" s="58" t="n"/>
+      <c r="K71" s="58" t="n"/>
+      <c r="L71" s="58" t="n"/>
+      <c r="M71" s="58" t="n"/>
+      <c r="N71" s="58" t="n"/>
+    </row>
+    <row r="72" ht="60" customHeight="1">
       <c r="A72" s="54" t="inlineStr">
         <is>
           <t>Tier 2</t>
@@ -3928,23 +4042,33 @@
           <t>工務店比較機能</t>
         </is>
       </c>
-      <c r="F72" s="53" t="inlineStr">
+      <c r="F72" s="28" t="inlineStr">
+        <is>
+          <t>2〜3社を選択して横並び比較表を表示。比較項目：坪単価・対応エリア・平屋実績・デザイン・断熱/耐震。比較画面下部に「まとめて資料請求」ボタン</t>
+        </is>
+      </c>
+      <c r="G72" s="53" t="inlineStr">
         <is>
           <t>CV率向上</t>
         </is>
       </c>
-      <c r="G72" s="53" t="inlineStr">
+      <c r="H72" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H72" s="53" t="inlineStr">
+      <c r="I72" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="73">
+      <c r="J72" s="58" t="n"/>
+      <c r="K72" s="58" t="n"/>
+      <c r="L72" s="58" t="n"/>
+      <c r="M72" s="58" t="n"/>
+      <c r="N72" s="58" t="n"/>
+    </row>
+    <row r="73" ht="60" customHeight="1">
       <c r="A73" s="54" t="inlineStr">
         <is>
           <t>Tier 2</t>
@@ -3970,23 +4094,33 @@
           <t>フィルター検索</t>
         </is>
       </c>
-      <c r="F73" s="53" t="inlineStr">
+      <c r="F73" s="28" t="inlineStr">
+        <is>
+          <t>工務店一覧にフィルターUI。項目：エリア・価格帯（〜1,500万/1,500〜2,500万/2,500万〜）・特徴（家事動線/中庭/ガレージ/コンパクト/バリアフリー）</t>
+        </is>
+      </c>
+      <c r="G73" s="53" t="inlineStr">
         <is>
           <t>UX向上</t>
         </is>
       </c>
-      <c r="G73" s="53" t="inlineStr">
+      <c r="H73" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H73" s="53" t="inlineStr">
+      <c r="I73" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="74">
+      <c r="J73" s="58" t="n"/>
+      <c r="K73" s="58" t="n"/>
+      <c r="L73" s="58" t="n"/>
+      <c r="M73" s="58" t="n"/>
+      <c r="N73" s="58" t="n"/>
+    </row>
+    <row r="74" ht="60" customHeight="1">
       <c r="A74" s="54" t="inlineStr">
         <is>
           <t>Tier 2</t>
@@ -4012,23 +4146,33 @@
           <t>お気に入り強化</t>
         </is>
       </c>
-      <c r="F74" s="53" t="inlineStr">
+      <c r="F74" s="28" t="inlineStr">
+        <is>
+          <t>お気に入り工務店が見学会を開催する際にメール通知を送信。「お気に入りの○○工務店が見学会を開催します」。再訪率・見学会予約率の向上</t>
+        </is>
+      </c>
+      <c r="G74" s="53" t="inlineStr">
         <is>
           <t>再訪率向上</t>
         </is>
       </c>
-      <c r="G74" s="53" t="inlineStr">
+      <c r="H74" s="53" t="inlineStr">
         <is>
           <t>3日</t>
         </is>
       </c>
-      <c r="H74" s="53" t="inlineStr">
+      <c r="I74" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="75">
+      <c r="J74" s="58" t="n"/>
+      <c r="K74" s="58" t="n"/>
+      <c r="L74" s="58" t="n"/>
+      <c r="M74" s="58" t="n"/>
+      <c r="N74" s="58" t="n"/>
+    </row>
+    <row r="75" ht="60" customHeight="1">
       <c r="A75" s="55" t="inlineStr">
         <is>
           <t>Tier 3</t>
@@ -4054,23 +4198,33 @@
           <t>消費者フォローメール自動配信</t>
         </is>
       </c>
-      <c r="F75" s="53" t="inlineStr">
+      <c r="F75" s="28" t="inlineStr">
+        <is>
+          <t>リード発生後9通の自動配信。3日後「連絡ありましたか？」→1週間後→1ヶ月後→3ヶ月後「ご契約は？」のアンケート付き。成約把握率を50%→85%に改善し回収漏れを防止</t>
+        </is>
+      </c>
+      <c r="G75" s="53" t="inlineStr">
         <is>
           <t>年間+500万円</t>
         </is>
       </c>
-      <c r="G75" s="53" t="inlineStr">
+      <c r="H75" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H75" s="53" t="inlineStr">
+      <c r="I75" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="76">
+      <c r="J75" s="58" t="n"/>
+      <c r="K75" s="58" t="n"/>
+      <c r="L75" s="58" t="n"/>
+      <c r="M75" s="58" t="n"/>
+      <c r="N75" s="58" t="n"/>
+    </row>
+    <row r="76" ht="60" customHeight="1">
       <c r="A76" s="55" t="inlineStr">
         <is>
           <t>Tier 3</t>
@@ -4096,23 +4250,33 @@
           <t>OBの声セクション</t>
         </is>
       </c>
-      <c r="F76" s="53" t="inlineStr">
+      <c r="F76" s="28" t="inlineStr">
+        <is>
+          <t>工務店詳細に「この工務店で建てた方の声」を追加。テキスト＋写真で3〜5件のOBレビュー。「建てて良かった」の声が成約の最後の一押し</t>
+        </is>
+      </c>
+      <c r="G76" s="53" t="inlineStr">
         <is>
           <t>成約率向上</t>
         </is>
       </c>
-      <c r="G76" s="53" t="inlineStr">
+      <c r="H76" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H76" s="53" t="inlineStr">
+      <c r="I76" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="77">
+      <c r="J76" s="58" t="n"/>
+      <c r="K76" s="58" t="n"/>
+      <c r="L76" s="58" t="n"/>
+      <c r="M76" s="58" t="n"/>
+      <c r="N76" s="58" t="n"/>
+    </row>
+    <row r="77" ht="60" customHeight="1">
       <c r="A77" s="55" t="inlineStr">
         <is>
           <t>Tier 3</t>
@@ -4138,23 +4302,33 @@
           <t>AIチャット→工務店推薦</t>
         </is>
       </c>
-      <c r="F77" s="53" t="inlineStr">
+      <c r="F77" s="28" t="inlineStr">
+        <is>
+          <t>会話中に「御社の条件なら○○工務店がおすすめです。今週末の見学会はいかがですか？」と推薦。エリア・予算・こだわりを抽出→フィルター→推薦生成</t>
+        </is>
+      </c>
+      <c r="G77" s="53" t="inlineStr">
         <is>
           <t>CV率向上</t>
         </is>
       </c>
-      <c r="G77" s="53" t="inlineStr">
+      <c r="H77" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H77" s="53" t="inlineStr">
+      <c r="I77" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="78">
+      <c r="J77" s="58" t="n"/>
+      <c r="K77" s="58" t="n"/>
+      <c r="L77" s="58" t="n"/>
+      <c r="M77" s="58" t="n"/>
+      <c r="N77" s="58" t="n"/>
+    </row>
+    <row r="78" ht="60" customHeight="1">
       <c r="A78" s="55" t="inlineStr">
         <is>
           <t>Tier 3</t>
@@ -4180,23 +4354,33 @@
           <t>見学会カレンダー表示</t>
         </is>
       </c>
-      <c r="F78" s="53" t="inlineStr">
+      <c r="F78" s="28" t="inlineStr">
+        <is>
+          <t>月間カレンダー形式で全工務店の見学会を一覧表示。日付クリックでその日の見学会一覧。「来週の土曜日どこかやってないかな」に対応</t>
+        </is>
+      </c>
+      <c r="G78" s="53" t="inlineStr">
         <is>
           <t>発見率向上</t>
         </is>
       </c>
-      <c r="G78" s="53" t="inlineStr">
+      <c r="H78" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H78" s="53" t="inlineStr">
+      <c r="I78" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="79">
+      <c r="J78" s="58" t="n"/>
+      <c r="K78" s="58" t="n"/>
+      <c r="L78" s="58" t="n"/>
+      <c r="M78" s="58" t="n"/>
+      <c r="N78" s="58" t="n"/>
+    </row>
+    <row r="79" ht="60" customHeight="1">
       <c r="A79" s="55" t="inlineStr">
         <is>
           <t>Tier 3</t>
@@ -4222,23 +4406,33 @@
           <t>LINE通知連携</t>
         </is>
       </c>
-      <c r="F79" s="53" t="inlineStr">
+      <c r="F79" s="28" t="inlineStr">
+        <is>
+          <t>リード発生時にLINE公式経由で工務店に通知。メールは見逃すがLINEはすぐ見る。LINE Messaging API使用。掲載プロの付加価値</t>
+        </is>
+      </c>
+      <c r="G79" s="53" t="inlineStr">
         <is>
           <t>対応速度向上</t>
         </is>
       </c>
-      <c r="G79" s="53" t="inlineStr">
+      <c r="H79" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H79" s="53" t="inlineStr">
+      <c r="I79" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="80">
+      <c r="J79" s="58" t="n"/>
+      <c r="K79" s="58" t="n"/>
+      <c r="L79" s="58" t="n"/>
+      <c r="M79" s="58" t="n"/>
+      <c r="N79" s="58" t="n"/>
+    </row>
+    <row r="80" ht="60" customHeight="1">
       <c r="A80" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4264,23 +4458,33 @@
           <t>GA4カスタムイベント</t>
         </is>
       </c>
-      <c r="F80" s="53" t="inlineStr">
+      <c r="F80" s="28" t="inlineStr">
+        <is>
+          <t>page_view/article_read/video_view/builder_detail_view/favorite_add/comparison_add/chat_start/reservation_submit等をGA4に送信</t>
+        </is>
+      </c>
+      <c r="G80" s="53" t="inlineStr">
         <is>
           <t>データ基盤</t>
         </is>
       </c>
-      <c r="G80" s="53" t="inlineStr">
+      <c r="H80" s="53" t="inlineStr">
         <is>
           <t>1週間</t>
         </is>
       </c>
-      <c r="H80" s="53" t="inlineStr">
+      <c r="I80" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="81">
+      <c r="J80" s="58" t="n"/>
+      <c r="K80" s="58" t="n"/>
+      <c r="L80" s="58" t="n"/>
+      <c r="M80" s="58" t="n"/>
+      <c r="N80" s="58" t="n"/>
+    </row>
+    <row r="81" ht="60" customHeight="1">
       <c r="A81" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4306,23 +4510,33 @@
           <t>ユーザーダッシュボード</t>
         </is>
       </c>
-      <c r="F81" s="53" t="inlineStr">
+      <c r="F81" s="28" t="inlineStr">
+        <is>
+          <t>マイページにお気に入り・閲覧履歴・相談履歴・資料請求履歴をライブデータ表示。Supabaseのfavorites/user_events/chat_sessionsから取得</t>
+        </is>
+      </c>
+      <c r="G81" s="53" t="inlineStr">
         <is>
           <t>ユーザー体験</t>
         </is>
       </c>
-      <c r="G81" s="53" t="inlineStr">
+      <c r="H81" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H81" s="53" t="inlineStr">
+      <c r="I81" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="82">
+      <c r="J81" s="58" t="n"/>
+      <c r="K81" s="58" t="n"/>
+      <c r="L81" s="58" t="n"/>
+      <c r="M81" s="58" t="n"/>
+      <c r="N81" s="58" t="n"/>
+    </row>
+    <row r="82" ht="60" customHeight="1">
       <c r="A82" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4348,23 +4562,33 @@
           <t>工務店ダッシュボード</t>
         </is>
       </c>
-      <c r="F82" s="53" t="inlineStr">
+      <c r="F82" s="28" t="inlineStr">
+        <is>
+          <t>月間PV・リード数・反響単価・前月比を工務店がログインして確認。リード一覧・ステータス更新・見学会管理・請求確認。掲載プロの主要付加価値</t>
+        </is>
+      </c>
+      <c r="G82" s="53" t="inlineStr">
         <is>
           <t>工務店向け付加価値</t>
         </is>
       </c>
-      <c r="G82" s="53" t="inlineStr">
+      <c r="H82" s="53" t="inlineStr">
         <is>
           <t>3週間</t>
         </is>
       </c>
-      <c r="H82" s="53" t="inlineStr">
+      <c r="I82" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="83">
+      <c r="J82" s="58" t="n"/>
+      <c r="K82" s="58" t="n"/>
+      <c r="L82" s="58" t="n"/>
+      <c r="M82" s="58" t="n"/>
+      <c r="N82" s="58" t="n"/>
+    </row>
+    <row r="83" ht="60" customHeight="1">
       <c r="A83" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4390,23 +4614,33 @@
           <t>CMS構造化データフォーム</t>
         </is>
       </c>
-      <c r="F83" s="53" t="inlineStr">
+      <c r="F83" s="28" t="inlineStr">
+        <is>
+          <t>エリア・価格帯・平屋比率・間取り傾向・デザイン・断熱/耐震・家事動線・中庭・子育て/老後向き・顧客像・強み/弱みを構造化入力</t>
+        </is>
+      </c>
+      <c r="G83" s="53" t="inlineStr">
         <is>
           <t>AI推薦の基盤</t>
         </is>
       </c>
-      <c r="G83" s="53" t="inlineStr">
+      <c r="H83" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H83" s="53" t="inlineStr">
+      <c r="I83" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="84">
+      <c r="J83" s="58" t="n"/>
+      <c r="K83" s="58" t="n"/>
+      <c r="L83" s="58" t="n"/>
+      <c r="M83" s="58" t="n"/>
+      <c r="N83" s="58" t="n"/>
+    </row>
+    <row r="84" ht="60" customHeight="1">
       <c r="A84" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4432,23 +4666,33 @@
           <t>AI意向抽出・会話要約</t>
         </is>
       </c>
-      <c r="F84" s="53" t="inlineStr">
+      <c r="F84" s="28" t="inlineStr">
+        <is>
+          <t>チャットログからinferred_intent・extracted_tags・conversation_summaryを自動生成。GPT-4oでバッチ処理。工務店への意向要約レポートの素材</t>
+        </is>
+      </c>
+      <c r="G84" s="53" t="inlineStr">
         <is>
           <t>AI高度化</t>
         </is>
       </c>
-      <c r="G84" s="53" t="inlineStr">
+      <c r="H84" s="53" t="inlineStr">
         <is>
           <t>3週間</t>
         </is>
       </c>
-      <c r="H84" s="53" t="inlineStr">
+      <c r="I84" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="85">
+      <c r="J84" s="58" t="n"/>
+      <c r="K84" s="58" t="n"/>
+      <c r="L84" s="58" t="n"/>
+      <c r="M84" s="58" t="n"/>
+      <c r="N84" s="58" t="n"/>
+    </row>
+    <row r="85" ht="60" customHeight="1">
       <c r="A85" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4474,23 +4718,33 @@
           <t>ユーザープロフィール登録</t>
         </is>
       </c>
-      <c r="F85" s="53" t="inlineStr">
+      <c r="F85" s="28" t="inlineStr">
+        <is>
+          <t>家族構成・年齢層・建築予定時期・土地有無・希望エリア・予算帯・デザイン志向・性能志向・検討フェーズを登録。user_profilesテーブル保存</t>
+        </is>
+      </c>
+      <c r="G85" s="53" t="inlineStr">
         <is>
           <t>AI推薦精度</t>
         </is>
       </c>
-      <c r="G85" s="53" t="inlineStr">
+      <c r="H85" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H85" s="53" t="inlineStr">
+      <c r="I85" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
-    </row>
-    <row r="86">
+      <c r="J85" s="58" t="n"/>
+      <c r="K85" s="58" t="n"/>
+      <c r="L85" s="58" t="n"/>
+      <c r="M85" s="58" t="n"/>
+      <c r="N85" s="58" t="n"/>
+    </row>
+    <row r="86" ht="60" customHeight="1">
       <c r="A86" s="56" t="inlineStr">
         <is>
           <t>Tier 4</t>
@@ -4516,32 +4770,49 @@
           <t>リード自動スコアリング</t>
         </is>
       </c>
-      <c r="F86" s="53" t="inlineStr">
+      <c r="F86" s="28" t="inlineStr">
+        <is>
+          <t>行動データ（PV数・滞在時間・お気に入り数・比較回数・チャット利用・資料請求有無）から0〜100点を自動算出。Hot/Warm/Coldランク付け</t>
+        </is>
+      </c>
+      <c r="G86" s="53" t="inlineStr">
         <is>
           <t>営業効率化</t>
         </is>
       </c>
-      <c r="G86" s="53" t="inlineStr">
+      <c r="H86" s="53" t="inlineStr">
         <is>
           <t>2週間</t>
         </is>
       </c>
-      <c r="H86" s="53" t="inlineStr">
+      <c r="I86" s="53" t="inlineStr">
         <is>
           <t>❌ 未着手</t>
         </is>
       </c>
+      <c r="J86" s="58" t="n"/>
+      <c r="K86" s="58" t="n"/>
+      <c r="L86" s="58" t="n"/>
+      <c r="M86" s="58" t="n"/>
+      <c r="N86" s="58" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="58" t="n"/>
+      <c r="B87" s="58" t="n"/>
+      <c r="C87" s="58" t="n"/>
+      <c r="D87" s="58" t="n"/>
+      <c r="E87" s="58" t="n"/>
+      <c r="F87" s="58" t="n"/>
+      <c r="G87" s="58" t="n"/>
+      <c r="H87" s="58" t="n"/>
+      <c r="I87" s="58" t="n"/>
+      <c r="J87" s="58" t="n"/>
+      <c r="K87" s="58" t="n"/>
+      <c r="L87" s="58" t="n"/>
+      <c r="M87" s="58" t="n"/>
+      <c r="N87" s="58" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A62:H62"/>
-    <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A3:I3"/>
-  </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D12:D21 D25:D34 D38:D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="無効な値" error="ステータスを選択してください" type="list">
       <formula1>"✅ 完了,🔧 進行中,⚠️ 部分的,❌ 未実装,📋 未着手"</formula1>

</xml_diff>